<commit_message>
Adiciona lançamento esquecido: Villa carlota (01/10/2026) e refaz totais
Reinsere o lançamento no grupo FRAIS VISITES e recalcula subtotal,
TOTAL GÉNÉRAL e MONTANT À REMBOURSER (1.691,59€).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vekb9ot43cCA3hzynoNKH6
</commit_message>
<xml_diff>
--- a/planilha/Notes de frais Lacs Italiens 27-09-26.xlsx
+++ b/planilha/Notes de frais Lacs Italiens 27-09-26.xlsx
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1180,77 +1180,84 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>01/10/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Villa carlota</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS VISITES</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t>02/10/2026</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>villa Melzi</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="n">
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>FRAIS VISITES</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Sous-total</t>
         </is>
       </c>
-      <c r="B32" s="8" t="n"/>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="9">
-        <f>SUM(D29:D31)</f>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="9">
+        <f>SUM(D29:D32)</f>
         <v/>
       </c>
-      <c r="E32" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="10" t="n"/>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="10" t="n"/>
+      <c r="E34" s="10" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
         </is>
       </c>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="7" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>27/09/2026</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>kipoint consigne 2 bagages</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
-        </is>
-      </c>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="7" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1260,82 +1267,89 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
+          <t>kipoint consigne 2 bagages</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
           <t>pane tulipane</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="n">
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="n">
         <v>17.75</v>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>FRAIS, TAXES DE SEJOUR, REPAS Accompagnateur</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>Sous-total</t>
         </is>
       </c>
-      <c r="B37" s="8" t="n"/>
-      <c r="C37" s="8" t="n"/>
-      <c r="D37" s="9">
-        <f>SUM(D35:D36)</f>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="9">
+        <f>SUM(D36:D37)</f>
         <v/>
       </c>
-      <c r="E37" s="8" t="n"/>
+      <c r="E38" s="8" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+      <c r="A39" s="10" t="n"/>
+      <c r="B39" s="10" t="n"/>
+      <c r="C39" s="10" t="n"/>
+      <c r="D39" s="10" t="n"/>
+      <c r="E39" s="10" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>NOTE DE FRAIS HORS SEJOUR</t>
         </is>
       </c>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="6" t="n"/>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="7" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>26/09/2026</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Pirelli guest House taxe séjour</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>NOTE DE FRAIS HORS SEJOUR</t>
-        </is>
-      </c>
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>27/09/2026</t>
+          <t>26/09/2026</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Rossopomodoro petit déjeuner guide</t>
+          <t>Pirelli guest House taxe séjour</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -1344,7 +1358,7 @@
         </is>
       </c>
       <c r="D41" s="3" t="n">
-        <v>3.9</v>
+        <v>9.5</v>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
@@ -1355,12 +1369,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>03/10/2026</t>
+          <t>27/09/2026</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>bar illy repas guide</t>
+          <t>Rossopomodoro petit déjeuner guide</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -1369,7 +1383,7 @@
         </is>
       </c>
       <c r="D42" s="3" t="n">
-        <v>20.1</v>
+        <v>3.9</v>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
@@ -1385,87 +1399,126 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
+          <t>bar illy repas guide</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>NOTE DE FRAIS HORS SEJOUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
           <t>Trenord como-milan</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="n">
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="n">
         <v>5.4</v>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>NOTE DE FRAIS HORS SEJOUR</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t>Sous-total</t>
         </is>
       </c>
-      <c r="B44" s="8" t="n"/>
-      <c r="C44" s="8" t="n"/>
-      <c r="D44" s="9">
-        <f>SUM(D40:D43)</f>
+      <c r="B45" s="8" t="n"/>
+      <c r="C45" s="8" t="n"/>
+      <c r="D45" s="9">
+        <f>SUM(D41:D44)</f>
         <v/>
       </c>
-      <c r="E44" s="8" t="n"/>
+      <c r="E45" s="8" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="11" t="inlineStr">
+      <c r="A46" s="10" t="n"/>
+      <c r="B46" s="10" t="n"/>
+      <c r="C46" s="10" t="n"/>
+      <c r="D46" s="10" t="n"/>
+      <c r="E46" s="10" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="11" t="inlineStr">
         <is>
           <t>TOTAL GÉNÉRAL</t>
         </is>
       </c>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="7" t="n"/>
-      <c r="D46" s="12">
-        <f>D15+D26+D32+D37+D44</f>
+      <c r="B47" s="6" t="n"/>
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="12">
+        <f>D15+D26+D33+D38+D45</f>
         <v/>
       </c>
-      <c r="E46" s="11" t="n"/>
+      <c r="E47" s="11" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="A48" s="10" t="n"/>
+      <c r="B48" s="10" t="n"/>
+      <c r="C48" s="10" t="n"/>
+      <c r="D48" s="10" t="n"/>
+      <c r="E48" s="10" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
         <is>
           <t>Avance reçue</t>
-        </is>
-      </c>
-      <c r="B48" s="6" t="n"/>
-      <c r="C48" s="7" t="n"/>
-      <c r="D48" s="14" t="n">
-        <v>-0</v>
-      </c>
-      <c r="E48" s="13" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="11" t="inlineStr">
-        <is>
-          <t>MONTANT À REMBOURSER</t>
         </is>
       </c>
       <c r="B49" s="6" t="n"/>
       <c r="C49" s="7" t="n"/>
-      <c r="D49" s="15">
-        <f>D46+D48</f>
+      <c r="D49" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="13" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>MONTANT À REMBOURSER</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="n"/>
+      <c r="C50" s="7" t="n"/>
+      <c r="D50" s="15">
+        <f>D47+D49</f>
         <v/>
       </c>
-      <c r="E49" s="11" t="n"/>
+      <c r="E50" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A35:E35"/>
     <mergeCell ref="A49:C49"/>
-    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A47:C47"/>
     <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A40:E40"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A50:C50"/>
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>

</xml_diff>